<commit_message>
Update website from Excel and improve synchronization script
</commit_message>
<xml_diff>
--- a/goods(4).xlsx
+++ b/goods(4).xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="108">
   <si>
     <t>Bags</t>
   </si>
@@ -225,6 +225,120 @@
   </si>
   <si>
     <t>Short Description</t>
+  </si>
+  <si>
+    <t>A handmade leather messenger bag designed for everyday carry, combining practical functionality, durable craftsmanship and timeless style</t>
+  </si>
+  <si>
+    <t>A minimalist handmade leather satchel designed for everyday work and travel, combining practical organization with timeless craftsmanship.</t>
+  </si>
+  <si>
+    <t>A compact handmade leather crossbody bag that combines everyday functionality, comfortable carry and a classic timeless design.</t>
+  </si>
+  <si>
+    <t>A versatile handmade genuine leather sling bag designed for convenient everyday carry with a minimalist and timeless look.</t>
+  </si>
+  <si>
+    <t>A handmade brown leather minimalist wallet designed to keep essential cards organized in a compact and practical everyday carry accessory.</t>
+  </si>
+  <si>
+    <t>A hand-sewn brown leather wallet crafted from premium Italian leather, combining classic craftsmanship with practical everyday organization.</t>
+  </si>
+  <si>
+    <t>A heavy-duty handmade black leather belt designed for everyday wear, featuring durable craftsmanship and a classic Italian buckle.</t>
+  </si>
+  <si>
+    <t>A handmade full-grain black leather belt designed for reliable everyday wear, with a classic silver buckle and durable construction.</t>
+  </si>
+  <si>
+    <t>A handmade full-grain black leather belt with a minimalist design, combining timeless style, durability and everyday functionality.</t>
+  </si>
+  <si>
+    <t>A durable handmade black leather work belt crafted from full-grain leather and designed for comfortable everyday use.</t>
+  </si>
+  <si>
+    <t>A classic handmade full-grain leather belt created for everyday wear, combining strong materials, practical design and timeless style.</t>
+  </si>
+  <si>
+    <t>A handmade black full-grain leather belt with a clean minimalist design, created as a durable and versatile everyday accessory.</t>
+  </si>
+  <si>
+    <t>A hand-stitched brown leather belt pouch designed for convenient EDC carry, keeping everyday essentials organized and easily accessible.</t>
+  </si>
+  <si>
+    <t>A handmade black leather belt pouch designed for practical everyday carry, combining durable craftsmanship with convenient organization.</t>
+  </si>
+  <si>
+    <t>A handmade leather EDC belt pouch designed to keep coins, cards and small everyday essentials organized and easy to access.</t>
+  </si>
+  <si>
+    <t>A handmade leather belt card holder designed for minimalist everyday carry, combining secure card storage with convenient belt-loop access.</t>
+  </si>
+  <si>
+    <t>A handmade leather belt pouch designed to organize coins, cards and small everyday essentials in a compact EDC accessory.</t>
+  </si>
+  <si>
+    <t>A handmade full-grain leather EDC belt pouch designed to keep coins, keys and everyday essentials organized and easily accessible.</t>
+  </si>
+  <si>
+    <t>Alt Text</t>
+  </si>
+  <si>
+    <t>Handmade gray leather messenger bag with a flap and shoulder strap displayed outdoors</t>
+  </si>
+  <si>
+    <t>Handmade black leather satchel crossbody bag with a flap and adjustable shoulder strap</t>
+  </si>
+  <si>
+    <t>Handmade gray leather crossbody messenger bag hanging from a tree outdoors</t>
+  </si>
+  <si>
+    <t>Handmade cognac brown leather sling bag worn across the back</t>
+  </si>
+  <si>
+    <t>Handmade brown leather minimalist wallet and card holder displayed with cards</t>
+  </si>
+  <si>
+    <t>Hand sewn brown leather wallet and coin holder resting on denim fabric</t>
+  </si>
+  <si>
+    <t>Heavy duty black leather belt with a large rectangular metal buckle</t>
+  </si>
+  <si>
+    <t>Handmade black full grain leather belt with a silver metal buckle</t>
+  </si>
+  <si>
+    <t>Handmade black leather belt with a minimalist rectangular metal buckle</t>
+  </si>
+  <si>
+    <t>Black full grain leather belt with a classic rectangular metal buckle</t>
+  </si>
+  <si>
+    <t>Handmade black leather belt with a silver rectangular buckle displayed on a light background</t>
+  </si>
+  <si>
+    <t>Handmade black full grain leather belt with a classic brass tone buckle</t>
+  </si>
+  <si>
+    <t>Hand stitched brown leather belt pouch worn on a belt with everyday carry gear</t>
+  </si>
+  <si>
+    <t>Handmade black leather belt pouch displayed with keys, cards and everyday carry items</t>
+  </si>
+  <si>
+    <t>Handmade brown leather belt pouch attached to a belt over denim jeans</t>
+  </si>
+  <si>
+    <t>Handmade brown leather belt card holder worn at the waist</t>
+  </si>
+  <si>
+    <t>Handmade brown leather belt pouch with flap closure worn on denim jeans</t>
+  </si>
+  <si>
+    <t>Handmade brown leather EDC pouch displayed with keys, cards and everyday carry accessories</t>
+  </si>
+  <si>
+    <t>SOLD</t>
   </si>
 </sst>
 </file>
@@ -609,18 +723,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="3" width="47.5703125" customWidth="1"/>
     <col min="4" max="4" width="49.85546875" customWidth="1"/>
-    <col min="5" max="5" width="28.85546875" customWidth="1"/>
-    <col min="6" max="6" width="10.42578125" customWidth="1"/>
-    <col min="7" max="7" width="11.42578125" customWidth="1"/>
+    <col min="5" max="6" width="28.85546875" customWidth="1"/>
+    <col min="7" max="7" width="10.42578125" customWidth="1"/>
+    <col min="8" max="8" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>38</v>
       </c>
@@ -637,21 +751,24 @@
         <v>67</v>
       </c>
       <c r="F1" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>4</v>
+      <c r="C2" t="s">
+        <v>70</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>5</v>
@@ -660,21 +777,24 @@
         <v>47</v>
       </c>
       <c r="F2" t="s">
-        <v>43</v>
+        <v>89</v>
       </c>
       <c r="G2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+      <c r="H2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>6</v>
+      <c r="C3" t="s">
+        <v>71</v>
       </c>
       <c r="D3" t="s">
         <v>7</v>
@@ -683,21 +803,24 @@
         <v>48</v>
       </c>
       <c r="F3" t="s">
-        <v>43</v>
+        <v>90</v>
       </c>
       <c r="G3" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+      <c r="H3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>8</v>
+      <c r="C4" t="s">
+        <v>72</v>
       </c>
       <c r="D4" t="s">
         <v>9</v>
@@ -706,21 +829,24 @@
         <v>49</v>
       </c>
       <c r="F4" t="s">
-        <v>43</v>
+        <v>91</v>
       </c>
       <c r="G4" t="s">
+        <v>43</v>
+      </c>
+      <c r="H4" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>10</v>
+      <c r="C5" t="s">
+        <v>73</v>
       </c>
       <c r="D5" t="s">
         <v>11</v>
@@ -729,21 +855,24 @@
         <v>46</v>
       </c>
       <c r="F5" t="s">
-        <v>43</v>
+        <v>92</v>
       </c>
       <c r="G5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+      <c r="H5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>12</v>
+      <c r="C6" t="s">
+        <v>74</v>
       </c>
       <c r="D6" t="s">
         <v>13</v>
@@ -752,21 +881,24 @@
         <v>50</v>
       </c>
       <c r="F6" t="s">
-        <v>43</v>
+        <v>93</v>
       </c>
       <c r="G6" t="s">
+        <v>43</v>
+      </c>
+      <c r="H6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>14</v>
+      <c r="C7" t="s">
+        <v>75</v>
       </c>
       <c r="D7" t="s">
         <v>15</v>
@@ -775,21 +907,24 @@
         <v>51</v>
       </c>
       <c r="F7" t="s">
-        <v>43</v>
+        <v>94</v>
       </c>
       <c r="G7" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+      <c r="H7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>16</v>
+      <c r="C8" t="s">
+        <v>76</v>
       </c>
       <c r="D8" t="s">
         <v>17</v>
@@ -798,21 +933,24 @@
         <v>52</v>
       </c>
       <c r="F8" t="s">
-        <v>43</v>
+        <v>95</v>
       </c>
       <c r="G8" t="s">
+        <v>43</v>
+      </c>
+      <c r="H8" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>18</v>
+      <c r="C9" t="s">
+        <v>77</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>19</v>
@@ -821,21 +959,24 @@
         <v>54</v>
       </c>
       <c r="F9" t="s">
-        <v>43</v>
+        <v>96</v>
       </c>
       <c r="G9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+      <c r="H9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>20</v>
+      <c r="C10" t="s">
+        <v>78</v>
       </c>
       <c r="D10" t="s">
         <v>21</v>
@@ -844,21 +985,24 @@
         <v>53</v>
       </c>
       <c r="F10" t="s">
-        <v>43</v>
+        <v>97</v>
       </c>
       <c r="G10" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+      <c r="H10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>18</v>
+      <c r="C11" t="s">
+        <v>79</v>
       </c>
       <c r="D11" t="s">
         <v>22</v>
@@ -867,21 +1011,24 @@
         <v>55</v>
       </c>
       <c r="F11" t="s">
-        <v>43</v>
+        <v>98</v>
       </c>
       <c r="G11" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+      <c r="H11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>18</v>
+      <c r="C12" t="s">
+        <v>80</v>
       </c>
       <c r="D12" t="s">
         <v>23</v>
@@ -890,21 +1037,24 @@
         <v>56</v>
       </c>
       <c r="F12" t="s">
-        <v>43</v>
+        <v>99</v>
       </c>
       <c r="G12" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+      <c r="H12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>24</v>
+      <c r="C13" t="s">
+        <v>81</v>
       </c>
       <c r="D13" t="s">
         <v>25</v>
@@ -913,21 +1063,24 @@
         <v>57</v>
       </c>
       <c r="F13" t="s">
-        <v>43</v>
+        <v>100</v>
       </c>
       <c r="G13" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+      <c r="H13" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>26</v>
+      <c r="C14" t="s">
+        <v>82</v>
       </c>
       <c r="D14" t="s">
         <v>27</v>
@@ -936,21 +1089,24 @@
         <v>58</v>
       </c>
       <c r="F14" t="s">
-        <v>43</v>
+        <v>101</v>
       </c>
       <c r="G14" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>107</v>
+      </c>
+      <c r="H14" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>28</v>
+      <c r="C15" t="s">
+        <v>83</v>
       </c>
       <c r="D15" t="s">
         <v>29</v>
@@ -959,21 +1115,24 @@
         <v>59</v>
       </c>
       <c r="F15" t="s">
-        <v>43</v>
+        <v>102</v>
       </c>
       <c r="G15" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+      <c r="H15" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>30</v>
+      <c r="C16" t="s">
+        <v>84</v>
       </c>
       <c r="D16" t="s">
         <v>31</v>
@@ -982,21 +1141,24 @@
         <v>60</v>
       </c>
       <c r="F16" t="s">
-        <v>43</v>
+        <v>103</v>
       </c>
       <c r="G16" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+      <c r="H16" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>32</v>
+      <c r="C17" t="s">
+        <v>85</v>
       </c>
       <c r="D17" t="s">
         <v>33</v>
@@ -1005,21 +1167,24 @@
         <v>61</v>
       </c>
       <c r="F17" t="s">
-        <v>43</v>
+        <v>104</v>
       </c>
       <c r="G17" t="s">
+        <v>43</v>
+      </c>
+      <c r="H17" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>34</v>
+      <c r="C18" t="s">
+        <v>86</v>
       </c>
       <c r="D18" t="s">
         <v>35</v>
@@ -1028,21 +1193,24 @@
         <v>62</v>
       </c>
       <c r="F18" t="s">
-        <v>43</v>
+        <v>105</v>
       </c>
       <c r="G18" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+      <c r="H18" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>36</v>
+      <c r="C19" t="s">
+        <v>87</v>
       </c>
       <c r="D19" t="s">
         <v>37</v>
@@ -1051,9 +1219,12 @@
         <v>63</v>
       </c>
       <c r="F19" t="s">
-        <v>43</v>
+        <v>106</v>
       </c>
       <c r="G19" t="s">
+        <v>43</v>
+      </c>
+      <c r="H19" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1063,6 +1234,7 @@
     <hyperlink ref="D9" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add product offers to JSON-LD
</commit_message>
<xml_diff>
--- a/goods(4).xlsx
+++ b/goods(4).xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="111">
   <si>
     <t>Bags</t>
   </si>
@@ -339,6 +339,15 @@
   </si>
   <si>
     <t>SOLD</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>Currency</t>
+  </si>
+  <si>
+    <t>USD</t>
   </si>
 </sst>
 </file>
@@ -407,7 +416,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -421,6 +430,10 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Гиперссылка" xfId="1" builtinId="8"/>
@@ -723,7 +736,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -732,9 +745,11 @@
     <col min="5" max="6" width="28.85546875" customWidth="1"/>
     <col min="7" max="7" width="10.42578125" customWidth="1"/>
     <col min="8" max="8" width="11.42578125" customWidth="1"/>
+    <col min="9" max="9" width="9.140625" style="10"/>
+    <col min="10" max="10" width="9.140625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>38</v>
       </c>
@@ -759,8 +774,14 @@
       <c r="H1" s="4" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="I1" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -785,8 +806,14 @@
       <c r="H2" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="I2" s="10">
+        <v>94</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -811,8 +838,14 @@
       <c r="H3" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="I3" s="10">
+        <v>97</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
@@ -837,8 +870,14 @@
       <c r="H4" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="I4" s="10">
+        <v>79</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -863,8 +902,14 @@
       <c r="H5" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="I5" s="10">
+        <v>69</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
@@ -889,8 +934,14 @@
       <c r="H6" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="I6" s="10">
+        <v>75</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>1</v>
       </c>
@@ -915,8 +966,14 @@
       <c r="H7" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="I7" s="10">
+        <v>39</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>2</v>
       </c>
@@ -941,8 +998,14 @@
       <c r="H8" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="I8" s="10">
+        <v>39</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
@@ -967,8 +1030,14 @@
       <c r="H9" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="I9" s="10">
+        <v>49</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>2</v>
       </c>
@@ -993,8 +1062,14 @@
       <c r="H10" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="I10" s="10">
+        <v>49</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>2</v>
       </c>
@@ -1019,8 +1094,14 @@
       <c r="H11" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="I11" s="10">
+        <v>49</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>2</v>
       </c>
@@ -1045,8 +1126,14 @@
       <c r="H12" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="I12" s="10">
+        <v>49</v>
+      </c>
+      <c r="J12" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>2</v>
       </c>
@@ -1071,8 +1158,14 @@
       <c r="H13" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="I13" s="10">
+        <v>49</v>
+      </c>
+      <c r="J13" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>3</v>
       </c>
@@ -1097,8 +1190,14 @@
       <c r="H14" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="I14" s="10">
+        <v>49</v>
+      </c>
+      <c r="J14" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>3</v>
       </c>
@@ -1123,8 +1222,14 @@
       <c r="H15" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="I15" s="10">
+        <v>69</v>
+      </c>
+      <c r="J15" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>3</v>
       </c>
@@ -1149,8 +1254,14 @@
       <c r="H16" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="I16" s="10">
+        <v>67</v>
+      </c>
+      <c r="J16" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>3</v>
       </c>
@@ -1175,8 +1286,14 @@
       <c r="H17" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="I17" s="10">
+        <v>59</v>
+      </c>
+      <c r="J17" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>3</v>
       </c>
@@ -1201,8 +1318,14 @@
       <c r="H18" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="I18" s="10">
+        <v>67</v>
+      </c>
+      <c r="J18" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>3</v>
       </c>
@@ -1226,6 +1349,12 @@
       </c>
       <c r="H19" t="s">
         <v>44</v>
+      </c>
+      <c r="I19" s="10">
+        <v>69</v>
+      </c>
+      <c r="J19" s="8" t="s">
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>